<commit_message>
feat: implement dispatch component and add user roles, RBAC permissions, and dynamic field configuration support
</commit_message>
<xml_diff>
--- a/Archive_Docs/data3.xlsx
+++ b/Archive_Docs/data3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\warehouse project\Archive_Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D86DCE3-F00F-4AAB-BF9E-5DFB79792C6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{742A1FAE-10F2-4DCC-B7F0-32046AE7C68B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="338" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6735" yWindow="4185" windowWidth="21600" windowHeight="11295" tabRatio="338" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MAIN BASE" sheetId="1" r:id="rId1"/>

</xml_diff>